<commit_message>
Make Shop tappable with Cement, Electrical, and Sanitaryware photos
Adds the provided photo sets for these 3 Shop subcategories under
assets/shop/, normalized to the same "N.png" naming used for Services
(zips and "1 (N).png" naming dropped). Tapping them inside the Shop
list now opens the same SubcategoryScreen grid used for Services;
other Shop items (Tools, Steel, Paint, Hardware, Water tanks) still
fall back to "Coming soon" since they don't have photos yet.

SubcategoryScreen now takes a full imagePathPrefix instead of a
services-only folder name, so it works for both assets/services/... and
assets/shop/... Also syncs the updated xlsx/data - Copy.xlsx (adds a
shop sheet with per-subcategory names, unused directly by the app
since images are self-labeled, but useful as the source of truth).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/xlsx/data - Copy.xlsx
+++ b/xlsx/data - Copy.xlsx
@@ -8,28 +8,62 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prazzol\pakka-homes\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E36D08E7-C457-40CD-B353-1DDD80F198F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFC14F7-893A-4123-927C-EDD58376BEB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="services" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="shop" sheetId="3" r:id="rId3"/>
-    <sheet name="rentals" sheetId="4" r:id="rId4"/>
-    <sheet name="bookings" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="shop" sheetId="3" r:id="rId4"/>
+    <sheet name="rentals" sheetId="4" r:id="rId5"/>
+    <sheet name="bookings" sheetId="5" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="407">
   <si>
     <t>🏠</t>
   </si>
@@ -1208,6 +1242,48 @@
   </si>
   <si>
     <t>Disinfection</t>
+  </si>
+  <si>
+    <t>Main Category,Subcategories</t>
+  </si>
+  <si>
+    <t>Construction,"New House Construction,Building Extension,Renovation,Demolition,Foundation Work,RCC / Concrete Work,Brick / Block Work,Roofing,Boundary Wall,Structural Repair,Site Preparation,Contractor Services"</t>
+  </si>
+  <si>
+    <t>Electrical,"New Wiring,Electrical Repair,Switch &amp; Socket Installation,Light &amp; Fan Installation,MCB / DB Installation,Earthing,Inverter / UPS,Generator,Solar Installation,CCTV Installation,Doorbell / Intercom,Electrical Inspection"</t>
+  </si>
+  <si>
+    <t>Cleaning,"House Cleaning,Deep Cleaning,Kitchen Cleaning,Bathroom Cleaning,Sofa Cleaning,Carpet Cleaning,Window / Glass Cleaning,Post-Construction Cleaning,Water Tank Cleaning,Office Cleaning,Move-in / Move-out Cleaning"</t>
+  </si>
+  <si>
+    <t>Mason,"Brick / Block Work,Plastering,Concrete Work,Floor Screeding,Tile Work,Wall Repair,Boundary Wall,Drainage Work,Bathroom Masonry,Kitchen Masonry,Paving / Interlocking"</t>
+  </si>
+  <si>
+    <t>Appliance Repair,"Refrigerator,Washing Machine,Air Conditioner,Television,Microwave / Oven,Water Heater / Geyser,Electric Stove,Dishwasher,Water Purifier,Exhaust Fan,Small Appliances,Installation &amp; Servicing"</t>
+  </si>
+  <si>
+    <t>Plumbing,"Leakage Repair,Pipe Installation,Drain Blockage,Bathroom Plumbing,Kitchen Plumbing,Tap / Faucet Repair,Toilet Repair,Water Tank Installation,Pump Installation / Repair,Water Heater / Geyser,Drainage,New Water Line"</t>
+  </si>
+  <si>
+    <t>Painting,"Interior Painting,Exterior Painting,Wall Repainting,Texture Painting,Waterproof Paint,Wood Painting / Polishing,Metal Painting,Ceiling Painting,Decorative Painting,Wallpaper Installation,Color Consultation"</t>
+  </si>
+  <si>
+    <t>Carpenter,"Furniture Repair,Custom Furniture,Door Repair / Installation,Window Repair,Wardrobe,Kitchen Cabinets,Modular Kitchen,Bed,Table / Desk,Shelves,Wooden Flooring,Polishing"</t>
+  </si>
+  <si>
+    <t>Waterproofing,"Roof Waterproofing,Terrace Waterproofing,Bathroom Waterproofing,Basement Waterproofing,Wall Dampness,Water Leakage,Tank Waterproofing,Balcony Waterproofing,Joint / Crack Sealing,Waterproof Coating"</t>
+  </si>
+  <si>
+    <t>1.generate me images for this tabs, for my service app, in grid format so that spiltable by ai…......</t>
+  </si>
+  <si>
+    <t>2.make the backgroud white…......</t>
+  </si>
+  <si>
+    <t>3.do not have borders in the images as they may disturb while splitting</t>
+  </si>
+  <si>
+    <t>Interior ,"Interior Design,3D Design,Modular Kitchen,Wardrobe,False Ceiling,Partition,TV Unit,Lighting Design,Flooring,Wallpaper,Curtains / Blinds,Furniture,Office Interior,Commercial Interior,Textile/upholstery,Biophillic Design"</t>
   </si>
 </sst>
 </file>
@@ -2050,6 +2126,85 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73AC22EE-18B4-4FAA-99A7-91AEF18A343F}">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C16" t="s">
+        <v>399</v>
+      </c>
+      <c r="D16" t="s">
+        <v>403</v>
+      </c>
+      <c r="E16" t="s">
+        <v>404</v>
+      </c>
+      <c r="F16" t="s">
+        <v>405</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06C9BE44-72D7-49C8-88A1-F1D8B6919E58}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2116,17 +2271,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B46C272C-4B94-4202-A378-A4A29DE0A3A1}">
-  <dimension ref="A1:AC14"/>
+  <dimension ref="A1:AH14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.08984375" style="2" customWidth="1"/>
     <col min="2" max="3" width="22.7265625" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="8.7265625" style="2"/>
+    <col min="4" max="33" width="8.7265625" style="2"/>
+    <col min="34" max="34" width="228.54296875" style="2" customWidth="1"/>
+    <col min="35" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -2134,7 +2291,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:29" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:34" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
@@ -2159,8 +2316,12 @@
       <c r="N2" s="3" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="3" spans="1:29" ht="58" x14ac:dyDescent="0.35">
+      <c r="AH2" s="3" cm="1">
+        <f t="array" aca="1" ref="AH2" ca="1">AH2:AH14="("&amp;B2&amp;","&amp;D2&amp;","&amp;F2&amp;","&amp;H2&amp;","&amp;J2&amp;","&amp;L2&amp;","&amp;N2&amp;","&amp;P2&amp;","&amp;R2&amp;","&amp;T2&amp;","&amp;V2&amp;","&amp;X2&amp;","&amp;Z2&amp;","&amp;AB2&amp;","&amp;AD2&amp;")"</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -2206,8 +2367,12 @@
       <c r="AB3" s="2" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="4" spans="1:29" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="AH3" s="3" t="str">
+        <f t="shared" ref="AH3:AH14" si="0">"("&amp;B3&amp;","&amp;D3&amp;","&amp;F3&amp;","&amp;H3&amp;","&amp;J3&amp;","&amp;L3&amp;","&amp;N3&amp;","&amp;P3&amp;","&amp;R3&amp;","&amp;T3&amp;","&amp;V3&amp;","&amp;X3&amp;","&amp;Z3&amp;","&amp;AB3&amp;","&amp;AD3&amp;")"</f>
+        <v>(Wires &amp; Cables,Switches &amp; Sockets,MCB &amp; DB,Distribution Boards,LED Lights,Ceiling Fans,Exhaust Fans,Conduits &amp; Accessories,Electrical Pipes,Plugs &amp; Adapters,Extension Boards,Electrical Protection,Inverters &amp; UPS,Electrical Accessories,)</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>143</v>
       </c>
@@ -2247,8 +2412,12 @@
       <c r="X4" s="3" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="5" spans="1:29" ht="58" x14ac:dyDescent="0.35">
+      <c r="AH4" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Western Toilets,Indian Toilets,Wash Basins,Pedestal Basins,Counter Basins,Urinals,Bathtubs,Shower Panels,Flush Tanks,Toilet Seats,Sanitary Accessories,Mirrors,,,)</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>144</v>
       </c>
@@ -2288,8 +2457,12 @@
       <c r="X5" s="2" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="6" spans="1:29" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="AH5" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Hand Tools,Power Tools,Measuring Tools,Cutting Tools,Drilling Tools,Grinding Tools,Construction Tools,Plumbing Tools,Electrical Tools,Painting Tools,Safety Tools &amp; Equipment,Tool Boxes,,,)</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>145</v>
       </c>
@@ -2332,8 +2505,12 @@
       <c r="Z6" s="3" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="7" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="AH6" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(TMT Bars,Structural Steel,Steel Pipes,GI Pipes,MS Pipes,Angle Steel,Channel Steel,Flat Bars,Steel Sheets,Roofing Sheets,Binding Wire,Steel Mesh,Steel Accessories,,)</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>146</v>
       </c>
@@ -2376,8 +2553,12 @@
       <c r="Z7" s="2" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="8" spans="1:29" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="AH7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Interior Paint,Exterior Paint,Primer,Wall Putty,Wood Paint,Metal Paint,Enamel Paint,Texture Paint,Waterproof Paint,Roof Paint,Spray Paint,Thinner &amp; Solvents,Paint Accessories,,)</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>147</v>
       </c>
@@ -2426,8 +2607,12 @@
       <c r="AC8" s="3" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="9" spans="1:29" ht="58" x14ac:dyDescent="0.35">
+      <c r="AH8" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Nails,Screws,Bolts &amp; Nuts,Washers,Hinges,Locks &amp; Latches,Door Handles,Cabinet Hardware,Brackets,Hooks,Chains,Fasteners,Adhesives,Sealants,)</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>148</v>
       </c>
@@ -2461,8 +2646,12 @@
       <c r="T9" s="2" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="10" spans="1:29" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="AH9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Plastic Water Tanks,HDPE Water Tanks,FRP Water Tanks,Overhead Water Tanks,Underground Water Tanks,Loft Tanks,Septic Tanks,Water Tank Accessories,Tank Fittings,Water Tank Stands,,,,,)</v>
+      </c>
+    </row>
+    <row r="10" spans="1:34" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>244</v>
       </c>
@@ -2496,8 +2685,12 @@
       <c r="T10" s="3" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="11" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="AH10" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(PVC Pipes,CPVC Pipes,HDPE Pipes,PPR Pipes,UPVC Pipes,Pipe Fittings,Valves,Taps &amp; Faucets,Drainage Fittings,Water Pumps,,,,,)</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>245</v>
       </c>
@@ -2528,8 +2721,12 @@
       <c r="R11" s="2" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="12" spans="1:29" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="AH11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Floor Tiles,Wall Tiles,Porcelain Tiles,Ceramic Tiles,Outdoor Tiles,Parking Tiles,Tile Adhesive,Tile Grout,Tile Accessories,,,,,,)</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>39</v>
       </c>
@@ -2554,8 +2751,12 @@
       <c r="N12" s="3" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="13" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="AH12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(CGI Sheets,Color Coated Sheets,Polycarbonate Sheets,Roofing Accessories,Gutters,Roofing Screws,Insulation,,,,,,,,)</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>246</v>
       </c>
@@ -2583,8 +2784,12 @@
       <c r="P13" s="2" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="14" spans="1:29" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="AH13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Waterproofing Chemicals,Concrete Admixtures,Tile Adhesive,Grout,Crack Fillers,Sealants,Epoxy,Repair Chemicals,,,,,,,)</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>247</v>
       </c>
@@ -2608,6 +2813,10 @@
       </c>
       <c r="N14" s="3" t="s">
         <v>285</v>
+      </c>
+      <c r="AH14" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>(Safety Helmets,Safety Shoes,Gloves,Safety Goggles,Reflective Vests,Face Masks,Safety Harnesses,,,,,,,,)</v>
       </c>
     </row>
   </sheetData>
@@ -2615,7 +2824,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D3E24FA-109E-4CD8-9375-58018C2F9EC1}">
   <dimension ref="A1:U16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3223,7 +3432,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CEEE6B2-995C-46B9-B725-B1E98A50FC8F}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>